<commit_message>
Update schema version in excel
</commit_message>
<xml_diff>
--- a/Excel for reference/BattINFO_converter_standard_Excel_version_1.1.16_filled.xlsx
+++ b/Excel for reference/BattINFO_converter_standard_Excel_version_1.1.16_filled.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\battinfoconverter\Excel for reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22267ADF-A8EE-4D26-BBF2-8244EEB0F8E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A18E38-7729-4762-8486-9172F7477CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1800" yWindow="6900" windowWidth="22320" windowHeight="11880" activeTab="1" xr2:uid="{1A6D523C-FE67-4F3F-AA9B-E9FEE83DA8F2}"/>
+    <workbookView xWindow="25710" yWindow="6180" windowWidth="22320" windowHeight="11880" xr2:uid="{1A6D523C-FE67-4F3F-AA9B-E9FEE83DA8F2}"/>
   </bookViews>
   <sheets>
     <sheet name="@Schema" sheetId="2" r:id="rId1"/>
@@ -1234,9 +1234,6 @@
     <t>hasElectrolyte-hasSolute-hasAdditive-hasConstituentB-schema:productID</t>
   </si>
   <si>
-    <t>1.1.15</t>
-  </si>
-  <si>
     <t>hasCase-hasComponentA-type|CellLid-hasCoating</t>
   </si>
   <si>
@@ -1274,6 +1271,9 @@
   </si>
   <si>
     <t>http://www.w3.org/2000/01/rdf-schema#</t>
+  </si>
+  <si>
+    <t>1.1.16</t>
   </si>
 </sst>
 </file>
@@ -2517,10 +2517,10 @@
     </row>
     <row r="10" spans="1:101">
       <c r="A10" s="32" t="s">
+        <v>402</v>
+      </c>
+      <c r="B10" s="33" t="s">
         <v>403</v>
-      </c>
-      <c r="B10" s="33" t="s">
-        <v>404</v>
       </c>
       <c r="C10" s="33" t="s">
         <v>9</v>
@@ -2538,7 +2538,7 @@
         <v>371</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>396</v>
+        <v>409</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>9</v>
@@ -5838,7 +5838,7 @@
         <v>10</v>
       </c>
       <c r="E138" s="32" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F138" s="34"/>
       <c r="G138" s="2"/>
@@ -6137,7 +6137,7 @@
         <v>10</v>
       </c>
       <c r="E139" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="140" spans="1:287" s="32" customFormat="1">
@@ -6154,7 +6154,7 @@
         <v>10</v>
       </c>
       <c r="E140" s="32" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F140" s="34"/>
       <c r="G140" s="2"/>
@@ -6453,7 +6453,7 @@
         <v>10</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="142" spans="1:287" s="32" customFormat="1">
@@ -6470,7 +6470,7 @@
         <v>10</v>
       </c>
       <c r="E142" s="68" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="F142" s="34"/>
       <c r="G142" s="2"/>
@@ -6769,7 +6769,7 @@
         <v>10</v>
       </c>
       <c r="E143" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="144" spans="1:287" s="32" customFormat="1">
@@ -7999,7 +7999,7 @@
         <v>271</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C150" s="4" t="s">
         <v>9</v>
@@ -9083,7 +9083,7 @@
         <v>278</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -9115,7 +9115,7 @@
         <v>285</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -9131,7 +9131,7 @@
         <v>288</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>
@@ -9439,10 +9439,10 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
+        <v>404</v>
+      </c>
+      <c r="B19" t="s">
         <v>405</v>
-      </c>
-      <c r="B19" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -9713,59 +9713,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <FolderType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <CultureName xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Leaders>
-    <IsNotebookLocked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Invited_Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Math_Settings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Self_Registration_Enabled xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Has_Leaders_Only_SectionGroup xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Member_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Member_Groups>
-    <Distribution_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <AppVersion xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <DefaultSectionNames xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Templates xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <NotebookType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <TeamsChannelId xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Invited_Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Is_Collaboration_Space_Locked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Teams_Channel_Section_Location xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Members>
-    <Owner xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Owner>
-    <LMS_Mappings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-    <_activity xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100F5BD758A7F2BF742ADB9291A93682A9E" ma:contentTypeVersion="31" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="0517f02299b6dbd064809d9c3f869e8a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="35345429-01ed-4d83-85b9-6cc21878d784" xmlns:ns4="53f86fb7-11c0-476e-bf8b-57768422e991" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a7ff6e993c77c55b2c02ebba747ae01b" ns3:_="" ns4:_="">
     <xsd:import namespace="35345429-01ed-4d83-85b9-6cc21878d784"/>
@@ -10162,6 +10109,59 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <FolderType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <CultureName xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Leaders>
+    <IsNotebookLocked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Invited_Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Math_Settings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Self_Registration_Enabled xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Has_Leaders_Only_SectionGroup xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Member_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Member_Groups>
+    <Distribution_Groups xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <AppVersion xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <DefaultSectionNames xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Templates xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <NotebookType xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <TeamsChannelId xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Invited_Leaders xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Is_Collaboration_Space_Locked xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Teams_Channel_Section_Location xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <Members xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Members>
+    <Owner xmlns="35345429-01ed-4d83-85b9-6cc21878d784">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Owner>
+    <LMS_Mappings xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+    <_activity xmlns="35345429-01ed-4d83-85b9-6cc21878d784" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -10172,16 +10172,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2D89A20-922B-4399-8A99-02ABCC3D1E33}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="35345429-01ed-4d83-85b9-6cc21878d784"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D716C96-A80E-4732-A5D3-9C77E88EE8CA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10200,6 +10190,16 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2D89A20-922B-4399-8A99-02ABCC3D1E33}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="35345429-01ed-4d83-85b9-6cc21878d784"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E85C156E-EE0C-426A-92B3-CAF84DB17690}">
   <ds:schemaRefs>

</xml_diff>